<commit_message>
soporte multi-año: índice y en variables, NodeAssignment por año, plotter actualizado
- timeseries: days_within_year, get_node_assignment con clave (y,d,t,elhd), get_extraction_goal por año
- functions: model.days → days_within_year, todas las variables/constraints/objetivo con índice y
- opt_model: var_index_order actualizado con y
- reader: NodeAssignment=3 columnas metadata (id, elhd_name, ex_node_name)
- printer: var_index_schema y var_axis_order con y en todos los índices
- json_plotter: loaders con _extract_ydt_simple (formato nuevo y→d→t y viejo roto d→t→_N),
  _filter_yd, _detect_years, loops de plots por (year, day), groupby para evitar duplicados

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH_costos_nuevos/Costo_fijo/Carga_on_board_fixed_3estaciones_P320kW/elmo_data.xlsx
+++ b/data/Escenarios_DCH_costos_nuevos/Costo_fijo/Carga_on_board_fixed_3estaciones_P320kW/elmo_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH_costos_nuevos\Costo_fijo\Carga_on_board_fixed_3estaciones_P320kW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Escenarios_DCH_costos_nuevos\Costo_fijo\Carga_on_board_fixed_3estaciones_P320kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6EAEB87-AD9E-4299-B7B9-B63E3B758104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -2087,36 +2087,36 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AD17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" style="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" style="21" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7" style="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="21" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" style="21" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="21" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.5703125" style="22" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.5546875" style="22" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="22" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.85546875" style="22" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.85546875" style="22" customWidth="1"/>
-    <col min="24" max="24" width="18.42578125" style="22" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" style="22" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="22" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.88671875" style="22" customWidth="1"/>
+    <col min="24" max="24" width="18.44140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.5546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.33203125" style="22" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="28" t="s">
         <v>3</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="29">
         <v>1</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="29">
         <v>2</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="29">
         <v>3</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="29">
         <v>4</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="29">
         <v>5</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="29">
         <v>6</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="29">
         <v>7</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="29">
         <v>8</v>
       </c>
@@ -3012,7 +3012,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="29">
         <v>9</v>
       </c>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="AD11"/>
     </row>
-    <row r="12" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="29">
         <v>10</v>
       </c>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="AD12"/>
     </row>
-    <row r="13" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="29">
         <v>11</v>
       </c>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="AD13"/>
     </row>
-    <row r="14" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="29">
         <v>12</v>
       </c>
@@ -3372,9 +3372,9 @@
       </c>
       <c r="AD14"/>
     </row>
-    <row r="15" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3384,17 +3384,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
-    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.44140625" customWidth="1"/>
+    <col min="7" max="7" width="21.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3533,9 +3533,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3606,17 +3606,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H346"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="48" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.140625" style="54" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="48" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.109375" style="54" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
@@ -3642,7 +3642,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="56" t="s">
         <v>3</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="57">
         <v>0</v>
       </c>
@@ -3694,7 +3694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="58">
         <v>1</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="58">
         <v>2</v>
       </c>
@@ -3746,7 +3746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="57">
         <v>3</v>
       </c>
@@ -3772,7 +3772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="58">
         <v>4</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="58">
         <v>5</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="57">
         <v>6</v>
       </c>
@@ -3850,7 +3850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="58">
         <v>7</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="58">
         <v>8</v>
       </c>
@@ -3902,7 +3902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="57">
         <v>9</v>
       </c>
@@ -3928,7 +3928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="58">
         <v>10</v>
       </c>
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="58">
         <v>11</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="58">
         <v>12</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="57">
         <v>13</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="58">
         <v>14</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="58">
         <v>15</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="57">
         <v>16</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="58">
         <v>17</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="58">
         <v>18</v>
       </c>
@@ -4162,7 +4162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="57">
         <v>19</v>
       </c>
@@ -4188,7 +4188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="58">
         <v>20</v>
       </c>
@@ -4214,7 +4214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="58">
         <v>21</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="58">
         <v>22</v>
       </c>
@@ -4266,7 +4266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="57">
         <v>23</v>
       </c>
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="58">
         <v>24</v>
       </c>
@@ -4318,7 +4318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="57">
         <v>25</v>
       </c>
@@ -4344,7 +4344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="58">
         <v>26</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="58">
         <v>27</v>
       </c>
@@ -4396,7 +4396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="57">
         <v>28</v>
       </c>
@@ -4422,7 +4422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="58">
         <v>29</v>
       </c>
@@ -4448,7 +4448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="58">
         <v>30</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="57">
         <v>31</v>
       </c>
@@ -4500,7 +4500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="58">
         <v>32</v>
       </c>
@@ -4526,7 +4526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="58">
         <v>33</v>
       </c>
@@ -4552,7 +4552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="57">
         <v>34</v>
       </c>
@@ -4578,7 +4578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="58">
         <v>35</v>
       </c>
@@ -4604,7 +4604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="58">
         <v>36</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="58">
         <v>37</v>
       </c>
@@ -4656,7 +4656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="57">
         <v>38</v>
       </c>
@@ -4682,7 +4682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="58">
         <v>39</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="58">
         <v>40</v>
       </c>
@@ -4734,7 +4734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="58">
         <v>41</v>
       </c>
@@ -4760,7 +4760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="58">
         <v>42</v>
       </c>
@@ -4786,7 +4786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="58">
         <v>43</v>
       </c>
@@ -4812,7 +4812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="58">
         <v>44</v>
       </c>
@@ -4838,7 +4838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="58">
         <v>45</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="58">
         <v>46</v>
       </c>
@@ -4890,7 +4890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="58">
         <v>47</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="58">
         <v>48</v>
       </c>
@@ -4942,7 +4942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="58">
         <v>49</v>
       </c>
@@ -4968,7 +4968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="58">
         <v>50</v>
       </c>
@@ -4994,7 +4994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="58">
         <v>51</v>
       </c>
@@ -5020,7 +5020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="58">
         <v>52</v>
       </c>
@@ -5046,7 +5046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="58">
         <v>53</v>
       </c>
@@ -5072,7 +5072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="58">
         <v>54</v>
       </c>
@@ -5098,7 +5098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="58">
         <v>55</v>
       </c>
@@ -5124,7 +5124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="58">
         <v>56</v>
       </c>
@@ -5150,7 +5150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="58">
         <v>57</v>
       </c>
@@ -5176,7 +5176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="58">
         <v>58</v>
       </c>
@@ -5202,7 +5202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="58">
         <v>59</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="58">
         <v>60</v>
       </c>
@@ -5254,7 +5254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="58">
         <v>61</v>
       </c>
@@ -5280,7 +5280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="58">
         <v>62</v>
       </c>
@@ -5306,7 +5306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="58">
         <v>63</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="58">
         <v>64</v>
       </c>
@@ -5358,7 +5358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="58">
         <v>65</v>
       </c>
@@ -5384,7 +5384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="58">
         <v>66</v>
       </c>
@@ -5410,7 +5410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="58">
         <v>67</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="58">
         <v>68</v>
       </c>
@@ -5462,7 +5462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="58">
         <v>69</v>
       </c>
@@ -5488,7 +5488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="58">
         <v>70</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="58">
         <v>71</v>
       </c>
@@ -5540,7 +5540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="58">
         <v>72</v>
       </c>
@@ -5566,7 +5566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="58">
         <v>73</v>
       </c>
@@ -5592,7 +5592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="58">
         <v>74</v>
       </c>
@@ -5618,7 +5618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="58">
         <v>75</v>
       </c>
@@ -5644,7 +5644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="58">
         <v>76</v>
       </c>
@@ -5670,7 +5670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="58">
         <v>77</v>
       </c>
@@ -5696,7 +5696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="58">
         <v>78</v>
       </c>
@@ -5722,7 +5722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="58">
         <v>79</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="58">
         <v>80</v>
       </c>
@@ -5774,7 +5774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="58">
         <v>81</v>
       </c>
@@ -5800,7 +5800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="58">
         <v>82</v>
       </c>
@@ -5826,7 +5826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="58">
         <v>83</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="58">
         <v>84</v>
       </c>
@@ -5878,7 +5878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="58">
         <v>85</v>
       </c>
@@ -5904,7 +5904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="58">
         <v>86</v>
       </c>
@@ -5930,7 +5930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="58">
         <v>87</v>
       </c>
@@ -5956,7 +5956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="58">
         <v>88</v>
       </c>
@@ -5982,7 +5982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="58">
         <v>89</v>
       </c>
@@ -6008,7 +6008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="58">
         <v>90</v>
       </c>
@@ -6034,7 +6034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="58">
         <v>91</v>
       </c>
@@ -6060,7 +6060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="58">
         <v>92</v>
       </c>
@@ -6086,7 +6086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="58">
         <v>93</v>
       </c>
@@ -6112,7 +6112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="58">
         <v>94</v>
       </c>
@@ -6138,7 +6138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="58">
         <v>95</v>
       </c>
@@ -6164,7 +6164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="58">
         <v>96</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="58">
         <v>97</v>
       </c>
@@ -6216,7 +6216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="58">
         <v>98</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="58">
         <v>99</v>
       </c>
@@ -6268,7 +6268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="58">
         <v>100</v>
       </c>
@@ -6294,7 +6294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="58">
         <v>101</v>
       </c>
@@ -6320,7 +6320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="58">
         <v>102</v>
       </c>
@@ -6346,7 +6346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="58">
         <v>103</v>
       </c>
@@ -6372,7 +6372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="58">
         <v>104</v>
       </c>
@@ -6398,7 +6398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="58">
         <v>105</v>
       </c>
@@ -6424,7 +6424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="58">
         <v>106</v>
       </c>
@@ -6450,7 +6450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="58">
         <v>107</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="58">
         <v>108</v>
       </c>
@@ -6502,7 +6502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="58">
         <v>109</v>
       </c>
@@ -6528,7 +6528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" s="58">
         <v>110</v>
       </c>
@@ -6554,7 +6554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" s="58">
         <v>111</v>
       </c>
@@ -6580,7 +6580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="58">
         <v>112</v>
       </c>
@@ -6606,7 +6606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="58">
         <v>113</v>
       </c>
@@ -6632,7 +6632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="58">
         <v>114</v>
       </c>
@@ -6658,7 +6658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="58">
         <v>115</v>
       </c>
@@ -6684,7 +6684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="58">
         <v>116</v>
       </c>
@@ -6710,7 +6710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="58">
         <v>117</v>
       </c>
@@ -6736,7 +6736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="58">
         <v>118</v>
       </c>
@@ -6762,7 +6762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="58">
         <v>119</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" s="58">
         <v>120</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" s="58">
         <v>121</v>
       </c>
@@ -6840,7 +6840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="58">
         <v>122</v>
       </c>
@@ -6866,7 +6866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="58">
         <v>123</v>
       </c>
@@ -6892,7 +6892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="58">
         <v>124</v>
       </c>
@@ -6918,7 +6918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="58">
         <v>125</v>
       </c>
@@ -6944,7 +6944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="58">
         <v>126</v>
       </c>
@@ -6970,7 +6970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" s="58">
         <v>127</v>
       </c>
@@ -6996,7 +6996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" s="58">
         <v>128</v>
       </c>
@@ -7022,7 +7022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" s="58">
         <v>129</v>
       </c>
@@ -7048,7 +7048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" s="58">
         <v>130</v>
       </c>
@@ -7074,7 +7074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="58">
         <v>131</v>
       </c>
@@ -7100,7 +7100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="58">
         <v>132</v>
       </c>
@@ -7126,7 +7126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" s="58">
         <v>133</v>
       </c>
@@ -7152,7 +7152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" s="58">
         <v>134</v>
       </c>
@@ -7178,7 +7178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" s="58">
         <v>135</v>
       </c>
@@ -7204,7 +7204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="58">
         <v>136</v>
       </c>
@@ -7230,7 +7230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" s="58">
         <v>137</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" s="58">
         <v>138</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" s="58">
         <v>139</v>
       </c>
@@ -7308,7 +7308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="58">
         <v>140</v>
       </c>
@@ -7334,7 +7334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" s="58">
         <v>141</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" s="58">
         <v>142</v>
       </c>
@@ -7386,7 +7386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="58">
         <v>143</v>
       </c>
@@ -7412,7 +7412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="58">
         <v>144</v>
       </c>
@@ -7438,7 +7438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="58">
         <v>145</v>
       </c>
@@ -7464,7 +7464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149" s="58">
         <v>146</v>
       </c>
@@ -7490,7 +7490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150" s="58">
         <v>147</v>
       </c>
@@ -7516,7 +7516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151" s="58">
         <v>148</v>
       </c>
@@ -7542,7 +7542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152" s="58">
         <v>149</v>
       </c>
@@ -7568,7 +7568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A153" s="58">
         <v>150</v>
       </c>
@@ -7594,7 +7594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A154" s="58">
         <v>151</v>
       </c>
@@ -7620,7 +7620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A155" s="58">
         <v>152</v>
       </c>
@@ -7646,7 +7646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156" s="58">
         <v>153</v>
       </c>
@@ -7672,7 +7672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A157" s="58">
         <v>154</v>
       </c>
@@ -7698,7 +7698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A158" s="58">
         <v>155</v>
       </c>
@@ -7724,7 +7724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A159" s="58">
         <v>156</v>
       </c>
@@ -7750,7 +7750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A160" s="58">
         <v>157</v>
       </c>
@@ -7776,7 +7776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A161" s="58">
         <v>158</v>
       </c>
@@ -7802,7 +7802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A162" s="58">
         <v>159</v>
       </c>
@@ -7828,7 +7828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A163" s="58">
         <v>160</v>
       </c>
@@ -7854,7 +7854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A164" s="58">
         <v>161</v>
       </c>
@@ -7880,7 +7880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A165" s="58">
         <v>162</v>
       </c>
@@ -7906,7 +7906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A166" s="58">
         <v>163</v>
       </c>
@@ -7932,7 +7932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A167" s="58">
         <v>164</v>
       </c>
@@ -7958,7 +7958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A168" s="58">
         <v>165</v>
       </c>
@@ -7984,7 +7984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A169" s="58">
         <v>166</v>
       </c>
@@ -8010,7 +8010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A170" s="58">
         <v>167</v>
       </c>
@@ -8036,7 +8036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A171" s="58">
         <v>168</v>
       </c>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A172" s="58">
         <v>169</v>
       </c>
@@ -8088,7 +8088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A173" s="58">
         <v>170</v>
       </c>
@@ -8114,7 +8114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A174" s="58">
         <v>171</v>
       </c>
@@ -8140,7 +8140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A175" s="58">
         <v>172</v>
       </c>
@@ -8166,7 +8166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A176" s="58">
         <v>173</v>
       </c>
@@ -8192,7 +8192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A177" s="58">
         <v>174</v>
       </c>
@@ -8218,7 +8218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A178" s="58">
         <v>175</v>
       </c>
@@ -8244,7 +8244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A179" s="58">
         <v>176</v>
       </c>
@@ -8270,7 +8270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A180" s="58">
         <v>177</v>
       </c>
@@ -8296,7 +8296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A181" s="58">
         <v>178</v>
       </c>
@@ -8322,7 +8322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A182" s="58">
         <v>179</v>
       </c>
@@ -8348,7 +8348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A183" s="58">
         <v>180</v>
       </c>
@@ -8374,7 +8374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A184" s="58">
         <v>181</v>
       </c>
@@ -8400,7 +8400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A185" s="58">
         <v>182</v>
       </c>
@@ -8426,7 +8426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A186" s="58">
         <v>183</v>
       </c>
@@ -8452,7 +8452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A187" s="58">
         <v>184</v>
       </c>
@@ -8478,7 +8478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A188" s="58">
         <v>185</v>
       </c>
@@ -8504,7 +8504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A189" s="58">
         <v>186</v>
       </c>
@@ -8530,7 +8530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A190" s="58">
         <v>187</v>
       </c>
@@ -8556,7 +8556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A191" s="58">
         <v>188</v>
       </c>
@@ -8582,7 +8582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A192" s="58">
         <v>189</v>
       </c>
@@ -8608,7 +8608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A193" s="58">
         <v>190</v>
       </c>
@@ -8634,7 +8634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A194" s="58">
         <v>191</v>
       </c>
@@ -8660,7 +8660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A195" s="58">
         <v>192</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A196" s="58">
         <v>193</v>
       </c>
@@ -8712,7 +8712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A197" s="58">
         <v>194</v>
       </c>
@@ -8738,7 +8738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A198" s="58">
         <v>195</v>
       </c>
@@ -8764,7 +8764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A199" s="58">
         <v>196</v>
       </c>
@@ -8790,7 +8790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A200" s="58">
         <v>197</v>
       </c>
@@ -8816,7 +8816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A201" s="58">
         <v>198</v>
       </c>
@@ -8842,7 +8842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A202" s="58">
         <v>199</v>
       </c>
@@ -8868,7 +8868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A203" s="58">
         <v>200</v>
       </c>
@@ -8894,7 +8894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A204" s="58">
         <v>201</v>
       </c>
@@ -8920,7 +8920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A205" s="58">
         <v>202</v>
       </c>
@@ -8946,7 +8946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A206" s="58">
         <v>203</v>
       </c>
@@ -8972,7 +8972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A207" s="58">
         <v>204</v>
       </c>
@@ -8998,7 +8998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A208" s="58">
         <v>205</v>
       </c>
@@ -9024,7 +9024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A209" s="58">
         <v>206</v>
       </c>
@@ -9050,7 +9050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A210" s="58">
         <v>207</v>
       </c>
@@ -9076,7 +9076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A211" s="58">
         <v>208</v>
       </c>
@@ -9102,7 +9102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A212" s="58">
         <v>209</v>
       </c>
@@ -9128,7 +9128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A213" s="58">
         <v>210</v>
       </c>
@@ -9154,7 +9154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A214" s="58">
         <v>211</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A215" s="58">
         <v>212</v>
       </c>
@@ -9206,7 +9206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A216" s="58">
         <v>213</v>
       </c>
@@ -9232,7 +9232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A217" s="58">
         <v>214</v>
       </c>
@@ -9258,7 +9258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A218" s="58">
         <v>215</v>
       </c>
@@ -9284,7 +9284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A219" s="58">
         <v>216</v>
       </c>
@@ -9310,7 +9310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A220" s="58">
         <v>217</v>
       </c>
@@ -9336,7 +9336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A221" s="58">
         <v>218</v>
       </c>
@@ -9362,7 +9362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A222" s="58">
         <v>219</v>
       </c>
@@ -9388,7 +9388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A223" s="58">
         <v>220</v>
       </c>
@@ -9414,7 +9414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A224" s="58">
         <v>221</v>
       </c>
@@ -9440,7 +9440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A225" s="58">
         <v>222</v>
       </c>
@@ -9466,7 +9466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A226" s="58">
         <v>223</v>
       </c>
@@ -9492,7 +9492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A227" s="58">
         <v>224</v>
       </c>
@@ -9518,7 +9518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A228" s="58">
         <v>225</v>
       </c>
@@ -9544,7 +9544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A229" s="58">
         <v>226</v>
       </c>
@@ -9570,7 +9570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A230" s="58">
         <v>227</v>
       </c>
@@ -9596,7 +9596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A231" s="58">
         <v>228</v>
       </c>
@@ -9622,7 +9622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A232" s="58">
         <v>229</v>
       </c>
@@ -9648,7 +9648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A233" s="58">
         <v>230</v>
       </c>
@@ -9674,7 +9674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A234" s="58">
         <v>231</v>
       </c>
@@ -9700,7 +9700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A235" s="58">
         <v>232</v>
       </c>
@@ -9726,7 +9726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A236" s="58">
         <v>233</v>
       </c>
@@ -9752,7 +9752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A237" s="58">
         <v>234</v>
       </c>
@@ -9778,7 +9778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A238" s="58">
         <v>235</v>
       </c>
@@ -9804,7 +9804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A239" s="58">
         <v>236</v>
       </c>
@@ -9830,7 +9830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A240" s="58">
         <v>237</v>
       </c>
@@ -9856,7 +9856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A241" s="58">
         <v>238</v>
       </c>
@@ -9882,7 +9882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A242" s="58">
         <v>239</v>
       </c>
@@ -9908,7 +9908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A243" s="58">
         <v>240</v>
       </c>
@@ -9934,7 +9934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A244" s="58">
         <v>241</v>
       </c>
@@ -9960,7 +9960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A245" s="58">
         <v>242</v>
       </c>
@@ -9986,7 +9986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A246" s="58">
         <v>243</v>
       </c>
@@ -10012,7 +10012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A247" s="58">
         <v>244</v>
       </c>
@@ -10038,7 +10038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A248" s="58">
         <v>245</v>
       </c>
@@ -10064,7 +10064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A249" s="58">
         <v>246</v>
       </c>
@@ -10090,7 +10090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A250" s="58">
         <v>247</v>
       </c>
@@ -10116,7 +10116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A251" s="58">
         <v>248</v>
       </c>
@@ -10142,7 +10142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A252" s="58">
         <v>249</v>
       </c>
@@ -10168,7 +10168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A253" s="58">
         <v>250</v>
       </c>
@@ -10194,7 +10194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A254" s="58">
         <v>251</v>
       </c>
@@ -10220,7 +10220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A255" s="58">
         <v>252</v>
       </c>
@@ -10246,7 +10246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A256" s="58">
         <v>253</v>
       </c>
@@ -10272,7 +10272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A257" s="58">
         <v>254</v>
       </c>
@@ -10298,7 +10298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A258" s="58">
         <v>255</v>
       </c>
@@ -10324,7 +10324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A259" s="58">
         <v>256</v>
       </c>
@@ -10350,7 +10350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A260" s="58">
         <v>257</v>
       </c>
@@ -10376,7 +10376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A261" s="58">
         <v>258</v>
       </c>
@@ -10402,7 +10402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A262" s="58">
         <v>259</v>
       </c>
@@ -10428,7 +10428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A263" s="58">
         <v>260</v>
       </c>
@@ -10454,7 +10454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A264" s="58">
         <v>261</v>
       </c>
@@ -10480,7 +10480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A265" s="58">
         <v>262</v>
       </c>
@@ -10506,7 +10506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A266" s="58">
         <v>263</v>
       </c>
@@ -10532,7 +10532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A267" s="58">
         <v>264</v>
       </c>
@@ -10558,7 +10558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A268" s="58">
         <v>265</v>
       </c>
@@ -10584,7 +10584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A269" s="58">
         <v>266</v>
       </c>
@@ -10610,7 +10610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A270" s="58">
         <v>267</v>
       </c>
@@ -10636,7 +10636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A271" s="58">
         <v>268</v>
       </c>
@@ -10662,7 +10662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A272" s="58">
         <v>269</v>
       </c>
@@ -10688,7 +10688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A273" s="58">
         <v>270</v>
       </c>
@@ -10714,7 +10714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A274" s="58">
         <v>271</v>
       </c>
@@ -10740,7 +10740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A275" s="58">
         <v>272</v>
       </c>
@@ -10766,7 +10766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A276" s="58">
         <v>273</v>
       </c>
@@ -10792,7 +10792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A277" s="58">
         <v>274</v>
       </c>
@@ -10818,7 +10818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A278" s="58">
         <v>275</v>
       </c>
@@ -10844,7 +10844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A279" s="58">
         <v>276</v>
       </c>
@@ -10870,7 +10870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A280" s="58">
         <v>277</v>
       </c>
@@ -10896,7 +10896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A281" s="58">
         <v>278</v>
       </c>
@@ -10922,7 +10922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A282" s="58">
         <v>279</v>
       </c>
@@ -10948,7 +10948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A283" s="58">
         <v>280</v>
       </c>
@@ -10974,7 +10974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A284" s="58">
         <v>281</v>
       </c>
@@ -11000,7 +11000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A285" s="58">
         <v>282</v>
       </c>
@@ -11026,7 +11026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A286" s="58">
         <v>283</v>
       </c>
@@ -11052,7 +11052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A287" s="58">
         <v>284</v>
       </c>
@@ -11078,7 +11078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A288" s="58">
         <v>285</v>
       </c>
@@ -11104,7 +11104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A289" s="58">
         <v>286</v>
       </c>
@@ -11130,7 +11130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A290" s="58">
         <v>287</v>
       </c>
@@ -11156,10 +11156,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A291" s="58"/>
     </row>
-    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A292" s="59"/>
       <c r="B292" s="69"/>
       <c r="C292" s="66"/>
@@ -11167,7 +11167,7 @@
       <c r="G292" s="39"/>
       <c r="H292" s="40"/>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A293" s="60"/>
       <c r="B293" s="69"/>
       <c r="C293" s="67"/>
@@ -11175,7 +11175,7 @@
       <c r="G293" s="35"/>
       <c r="H293" s="6"/>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A294" s="61"/>
       <c r="B294" s="69"/>
       <c r="C294" s="67"/>
@@ -11183,7 +11183,7 @@
       <c r="G294" s="35"/>
       <c r="H294" s="6"/>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A295" s="62"/>
       <c r="B295" s="69"/>
       <c r="C295" s="67"/>
@@ -11191,7 +11191,7 @@
       <c r="G295" s="35"/>
       <c r="H295" s="6"/>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A296" s="62"/>
       <c r="B296" s="69"/>
       <c r="C296" s="67"/>
@@ -11199,7 +11199,7 @@
       <c r="G296" s="35"/>
       <c r="H296" s="6"/>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A297" s="62"/>
       <c r="B297" s="69"/>
       <c r="C297" s="67"/>
@@ -11207,7 +11207,7 @@
       <c r="G297" s="35"/>
       <c r="H297" s="6"/>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A298" s="60"/>
       <c r="B298" s="69"/>
       <c r="C298" s="67"/>
@@ -11215,7 +11215,7 @@
       <c r="G298" s="35"/>
       <c r="H298" s="6"/>
     </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A299" s="61"/>
       <c r="B299" s="69"/>
       <c r="C299" s="67"/>
@@ -11223,7 +11223,7 @@
       <c r="G299" s="35"/>
       <c r="H299" s="6"/>
     </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A300" s="62"/>
       <c r="B300" s="69"/>
       <c r="C300" s="67"/>
@@ -11231,7 +11231,7 @@
       <c r="G300" s="35"/>
       <c r="H300" s="6"/>
     </row>
-    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A301" s="62"/>
       <c r="B301" s="69"/>
       <c r="C301" s="67"/>
@@ -11239,7 +11239,7 @@
       <c r="G301" s="35"/>
       <c r="H301" s="6"/>
     </row>
-    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A302" s="62"/>
       <c r="B302" s="69"/>
       <c r="C302" s="67"/>
@@ -11247,7 +11247,7 @@
       <c r="G302" s="35"/>
       <c r="H302" s="6"/>
     </row>
-    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A303" s="60"/>
       <c r="B303" s="69"/>
       <c r="C303" s="67"/>
@@ -11255,7 +11255,7 @@
       <c r="G303" s="35"/>
       <c r="H303" s="6"/>
     </row>
-    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A304" s="61"/>
       <c r="B304" s="69"/>
       <c r="C304" s="67"/>
@@ -11263,7 +11263,7 @@
       <c r="G304" s="35"/>
       <c r="H304" s="6"/>
     </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A305" s="62"/>
       <c r="B305" s="69"/>
       <c r="C305" s="67"/>
@@ -11271,7 +11271,7 @@
       <c r="G305" s="35"/>
       <c r="H305" s="6"/>
     </row>
-    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A306" s="62"/>
       <c r="B306" s="69"/>
       <c r="C306" s="67"/>
@@ -11279,7 +11279,7 @@
       <c r="G306" s="35"/>
       <c r="H306" s="6"/>
     </row>
-    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A307" s="62"/>
       <c r="B307" s="69"/>
       <c r="C307" s="67"/>
@@ -11287,7 +11287,7 @@
       <c r="G307" s="35"/>
       <c r="H307" s="6"/>
     </row>
-    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A308" s="60"/>
       <c r="B308" s="69"/>
       <c r="C308" s="67"/>
@@ -11295,7 +11295,7 @@
       <c r="G308" s="35"/>
       <c r="H308" s="6"/>
     </row>
-    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A309" s="61"/>
       <c r="B309" s="69"/>
       <c r="C309" s="67"/>
@@ -11303,7 +11303,7 @@
       <c r="G309" s="35"/>
       <c r="H309" s="6"/>
     </row>
-    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A310" s="62"/>
       <c r="B310" s="69"/>
       <c r="C310" s="67"/>
@@ -11311,7 +11311,7 @@
       <c r="G310" s="35"/>
       <c r="H310" s="6"/>
     </row>
-    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A311" s="62"/>
       <c r="B311" s="69"/>
       <c r="C311" s="67"/>
@@ -11319,7 +11319,7 @@
       <c r="G311" s="35"/>
       <c r="H311" s="6"/>
     </row>
-    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A312" s="62"/>
       <c r="B312" s="69"/>
       <c r="C312" s="67"/>
@@ -11327,7 +11327,7 @@
       <c r="G312" s="35"/>
       <c r="H312" s="6"/>
     </row>
-    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A313" s="60"/>
       <c r="B313" s="69"/>
       <c r="C313" s="67"/>
@@ -11335,7 +11335,7 @@
       <c r="G313" s="35"/>
       <c r="H313" s="6"/>
     </row>
-    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A314" s="61"/>
       <c r="B314" s="69"/>
       <c r="C314" s="67"/>
@@ -11343,7 +11343,7 @@
       <c r="G314" s="35"/>
       <c r="H314" s="6"/>
     </row>
-    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A315" s="62"/>
       <c r="B315" s="69"/>
       <c r="C315" s="67"/>
@@ -11351,7 +11351,7 @@
       <c r="G315" s="35"/>
       <c r="H315" s="6"/>
     </row>
-    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A316" s="62"/>
       <c r="B316" s="69"/>
       <c r="C316" s="67"/>
@@ -11359,7 +11359,7 @@
       <c r="G316" s="35"/>
       <c r="H316" s="6"/>
     </row>
-    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A317" s="62"/>
       <c r="B317" s="69"/>
       <c r="C317" s="67"/>
@@ -11367,7 +11367,7 @@
       <c r="G317" s="35"/>
       <c r="H317" s="6"/>
     </row>
-    <row r="318" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A318" s="60"/>
       <c r="B318" s="69"/>
       <c r="C318" s="67"/>
@@ -11375,7 +11375,7 @@
       <c r="G318" s="35"/>
       <c r="H318" s="6"/>
     </row>
-    <row r="319" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A319" s="61"/>
       <c r="B319" s="69"/>
       <c r="C319" s="67"/>
@@ -11383,7 +11383,7 @@
       <c r="G319" s="35"/>
       <c r="H319" s="6"/>
     </row>
-    <row r="320" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A320" s="62"/>
       <c r="B320" s="69"/>
       <c r="C320" s="67"/>
@@ -11391,7 +11391,7 @@
       <c r="G320" s="35"/>
       <c r="H320" s="6"/>
     </row>
-    <row r="321" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A321" s="62"/>
       <c r="B321" s="69"/>
       <c r="C321" s="67"/>
@@ -11399,7 +11399,7 @@
       <c r="G321" s="35"/>
       <c r="H321" s="6"/>
     </row>
-    <row r="322" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A322" s="62"/>
       <c r="B322" s="69"/>
       <c r="C322" s="67"/>
@@ -11407,7 +11407,7 @@
       <c r="G322" s="35"/>
       <c r="H322" s="6"/>
     </row>
-    <row r="323" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A323" s="60"/>
       <c r="B323" s="69"/>
       <c r="C323" s="67"/>
@@ -11415,7 +11415,7 @@
       <c r="G323" s="35"/>
       <c r="H323" s="6"/>
     </row>
-    <row r="324" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A324" s="61"/>
       <c r="B324" s="69"/>
       <c r="C324" s="67"/>
@@ -11423,7 +11423,7 @@
       <c r="G324" s="35"/>
       <c r="H324" s="6"/>
     </row>
-    <row r="325" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A325" s="62"/>
       <c r="B325" s="69"/>
       <c r="C325" s="67"/>
@@ -11431,7 +11431,7 @@
       <c r="G325" s="35"/>
       <c r="H325" s="6"/>
     </row>
-    <row r="326" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A326" s="62"/>
       <c r="B326" s="69"/>
       <c r="C326" s="67"/>
@@ -11439,7 +11439,7 @@
       <c r="G326" s="35"/>
       <c r="H326" s="6"/>
     </row>
-    <row r="327" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A327" s="62"/>
       <c r="B327" s="69"/>
       <c r="C327" s="67"/>
@@ -11447,7 +11447,7 @@
       <c r="G327" s="35"/>
       <c r="H327" s="6"/>
     </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A328" s="60"/>
       <c r="B328" s="69"/>
       <c r="C328" s="67"/>
@@ -11455,7 +11455,7 @@
       <c r="G328" s="35"/>
       <c r="H328" s="6"/>
     </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A329" s="61"/>
       <c r="B329" s="69"/>
       <c r="C329" s="67"/>
@@ -11463,7 +11463,7 @@
       <c r="G329" s="35"/>
       <c r="H329" s="6"/>
     </row>
-    <row r="330" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A330" s="62"/>
       <c r="B330" s="69"/>
       <c r="C330" s="67"/>
@@ -11471,7 +11471,7 @@
       <c r="G330" s="35"/>
       <c r="H330" s="6"/>
     </row>
-    <row r="331" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A331" s="62"/>
       <c r="B331" s="69"/>
       <c r="C331" s="67"/>
@@ -11479,7 +11479,7 @@
       <c r="G331" s="35"/>
       <c r="H331" s="6"/>
     </row>
-    <row r="332" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A332" s="62"/>
       <c r="B332" s="69"/>
       <c r="C332" s="67"/>
@@ -11487,7 +11487,7 @@
       <c r="G332" s="35"/>
       <c r="H332" s="6"/>
     </row>
-    <row r="333" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A333" s="60"/>
       <c r="B333" s="69"/>
       <c r="C333" s="67"/>
@@ -11495,7 +11495,7 @@
       <c r="G333" s="35"/>
       <c r="H333" s="6"/>
     </row>
-    <row r="334" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A334" s="61"/>
       <c r="B334" s="69"/>
       <c r="C334" s="67"/>
@@ -11503,7 +11503,7 @@
       <c r="G334" s="35"/>
       <c r="H334" s="6"/>
     </row>
-    <row r="335" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A335" s="62"/>
       <c r="B335" s="69"/>
       <c r="C335" s="67"/>
@@ -11511,7 +11511,7 @@
       <c r="G335" s="35"/>
       <c r="H335" s="6"/>
     </row>
-    <row r="336" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A336" s="62"/>
       <c r="B336" s="69"/>
       <c r="C336" s="67"/>
@@ -11519,7 +11519,7 @@
       <c r="G336" s="35"/>
       <c r="H336" s="6"/>
     </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A337" s="62"/>
       <c r="B337" s="69"/>
       <c r="C337" s="67"/>
@@ -11527,7 +11527,7 @@
       <c r="G337" s="35"/>
       <c r="H337" s="6"/>
     </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A338" s="60"/>
       <c r="B338" s="69"/>
       <c r="C338" s="67"/>
@@ -11535,7 +11535,7 @@
       <c r="G338" s="35"/>
       <c r="H338" s="6"/>
     </row>
-    <row r="339" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A339" s="61"/>
       <c r="B339" s="69"/>
       <c r="C339" s="67"/>
@@ -11543,7 +11543,7 @@
       <c r="G339" s="35"/>
       <c r="H339" s="6"/>
     </row>
-    <row r="340" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A340" s="62"/>
       <c r="B340" s="69"/>
       <c r="C340" s="67"/>
@@ -11551,7 +11551,7 @@
       <c r="G340" s="35"/>
       <c r="H340" s="6"/>
     </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A341" s="62"/>
       <c r="B341" s="69"/>
       <c r="C341" s="67"/>
@@ -11559,7 +11559,7 @@
       <c r="G341" s="35"/>
       <c r="H341" s="6"/>
     </row>
-    <row r="342" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A342" s="62"/>
       <c r="B342" s="69"/>
       <c r="C342" s="67"/>
@@ -11567,7 +11567,7 @@
       <c r="G342" s="35"/>
       <c r="H342" s="6"/>
     </row>
-    <row r="343" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A343" s="60"/>
       <c r="B343" s="69"/>
       <c r="C343" s="67"/>
@@ -11575,7 +11575,7 @@
       <c r="G343" s="35"/>
       <c r="H343" s="6"/>
     </row>
-    <row r="344" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A344" s="61"/>
       <c r="B344" s="69"/>
       <c r="C344" s="67"/>
@@ -11583,7 +11583,7 @@
       <c r="G344" s="35"/>
       <c r="H344" s="6"/>
     </row>
-    <row r="345" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A345" s="62"/>
       <c r="B345" s="69"/>
       <c r="C345" s="67"/>
@@ -11591,7 +11591,7 @@
       <c r="G345" s="35"/>
       <c r="H345" s="6"/>
     </row>
-    <row r="346" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A346" s="62"/>
       <c r="B346" s="69"/>
       <c r="C346" s="67"/>
@@ -11611,14 +11611,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -11629,7 +11629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -11640,7 +11640,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>0</v>
       </c>

</xml_diff>